<commit_message>
clarify(onboarding): stock options = number of shares, not 100-share contracts
User raised the right ambiguity: 'Options' could be read as exchange-traded contracts (1 contract = 100
shares). For EMPLOYEE equity comp the unit is the number of options (= shares), which is what we capture
and value at (market − strike) — correct, no ×100. Added a hint under the options input: 'Each option =
1 share — enter your grant count, NOT 100-share trading contracts.' Guard test pins it.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-test-plan-v1.0.8.xlsx
+++ b/docs/finwise-test-plan-v1.0.8.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36ADA282-0ADB-654A-8C59-204FFBE05BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9360BA-4716-9642-B3C7-1F59A436E822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="0" windowWidth="30440" windowHeight="10380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="0" windowWidth="30440" windowHeight="19580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to test" sheetId="1" r:id="rId1"/>
     <sheet name="Test cases" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Test cases'!A1:H31</definedName>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="193">
   <si>
     <t>FinWise — Device Test Plan (build 1.0.8)</t>
   </si>
@@ -534,6 +535,75 @@
   </si>
   <si>
     <t>income 4 of 12 is still 401K contributions</t>
+  </si>
+  <si>
+    <t>Onboarding</t>
+  </si>
+  <si>
+    <t>Income 6 of 12</t>
+  </si>
+  <si>
+    <t>Flow Tested</t>
+  </si>
+  <si>
+    <t>Annual bonus = $25000 paid in Dec</t>
+  </si>
+  <si>
+    <t>base salary = 25000</t>
+  </si>
+  <si>
+    <t>401K contribution = 1500</t>
+  </si>
+  <si>
+    <t>employer match = 50%</t>
+  </si>
+  <si>
+    <t>Equity-based compensation - stock options (strike price 25, market price 26); vesting schedule = 100 in june'26, 200 in Nov'26, 500 in Feb'27</t>
+  </si>
+  <si>
+    <t>self-employment income per year = 25000</t>
+  </si>
+  <si>
+    <t>Interest &amp; dividends = 35000 annual</t>
+  </si>
+  <si>
+    <t>rental property -&gt; short-term, avg rent/mo = 3000, operating expense/mo = 2500</t>
+  </si>
+  <si>
+    <t>Monthly/Annual</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>annual</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>add in dec</t>
+  </si>
+  <si>
+    <t>desired cash flow treatment</t>
+  </si>
+  <si>
+    <t>add monthly</t>
+  </si>
+  <si>
+    <t>Add in june and nov cash flow for 2026</t>
+  </si>
+  <si>
+    <t>divide monthly</t>
+  </si>
+  <si>
+    <t>App Cash Flow Treatment</t>
+  </si>
+  <si>
+    <t>divided montly</t>
+  </si>
+  <si>
+    <t>added monthly</t>
   </si>
 </sst>
 </file>
@@ -549,12 +619,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -569,9 +645,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1210,7 +1289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1522,7 +1601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>113</v>
       </c>
@@ -1756,7 +1835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>156</v>
       </c>
@@ -1782,7 +1861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>161</v>
       </c>
@@ -1815,4 +1894,154 @@
     <ignoredError sqref="A1:H1 A4:H9 A2:F2 H2 A3:F3 A11:H11 A10:F10 A13:H31 A12:D12 F12 H12" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FE6258-7A6E-E345-B240-956A6BDCE0B8}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="38.33203125" customWidth="1"/>
+    <col min="3" max="3" width="80.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="32.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C3" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C4" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C7" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C8" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C9" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(T19/#12): CSV import broke because readAsStringAsync THROWS (deprecated), not encoding
The diagnostic detail I added surfaced the true cause: expo-file-system's top-level readAsStringAsync is
deprecated in SDK 56 and throws at runtime — 'We couldn't read that file'. The jest mock hid it
(source-pass != device-pass). Fix: one canonical readFileString() wrapper over expo-file-system/legacy
(Expo's documented supported path); ImportHoldingsScreen + BudgetScreen route through it. jest now mocks
expo-file-system/legacy so tests exercise the real path. Verified by the production bundle (expo
export:embed) building clean. The base64/UTF-16 decode work still rides on top.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-test-plan-v1.0.8.xlsx
+++ b/docs/finwise-test-plan-v1.0.8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9360BA-4716-9642-B3C7-1F59A436E822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589C801A-ACA4-5443-A688-CEB04C364CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="0" windowWidth="30440" windowHeight="19580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to test" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="201">
   <si>
     <t>FinWise — Device Test Plan (build 1.0.8)</t>
   </si>
@@ -604,6 +604,30 @@
   </si>
   <si>
     <t>added monthly</t>
+  </si>
+  <si>
+    <t>when click on cash flow details it comes back to same screen</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Net worth setup flow asks for Cash, Investments, Property &amp; Debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net worth Donus list investment as Stock/ETF. No where we are explaining what's included in investment, versus Cash/Cash Equivalent versus Real Estate and Property. 401K/Roth = Unclassified. At the top of the donut we should explain asset classes. </t>
+  </si>
+  <si>
+    <t>We couldn't read that file. Your data is safe - try exporting a csv from your brokerage and pick it again. (Details: Method readAsStringAsync imported from "expo-file-system" is deprecated. You can migrate to the new filesystem API using "File" and "Directo)</t>
+  </si>
+  <si>
+    <t>Import is on NW screen. But the box need to be organized logically. Box currently says - Import, Portfolio, Bonds, Other investments (non-compliant with taxonomy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home screen Cash-Flow box still labels it as Left-over versus surplus. </t>
+  </si>
+  <si>
+    <t>only see the language on "stree test an emergency" screen.</t>
   </si>
 </sst>
 </file>
@@ -1256,14 +1280,14 @@
       <c r="F7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G7" t="s">
-        <v>1</v>
+      <c r="G7" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="H7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1282,11 +1306,11 @@
       <c r="F8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G8" t="s">
-        <v>1</v>
-      </c>
-      <c r="H8" t="s">
-        <v>1</v>
+      <c r="G8" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1308,8 +1332,8 @@
       <c r="F9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G9" t="s">
-        <v>1</v>
+      <c r="G9" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="H9" t="s">
         <v>1</v>
@@ -1360,8 +1384,8 @@
       <c r="F11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G11" t="s">
-        <v>1</v>
+      <c r="G11" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="H11" t="s">
         <v>1</v>
@@ -1412,14 +1436,14 @@
       <c r="F13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G13" t="s">
-        <v>1</v>
+      <c r="G13" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="H13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="187" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -1441,8 +1465,8 @@
       <c r="G14" t="s">
         <v>1</v>
       </c>
-      <c r="H14" t="s">
-        <v>1</v>
+      <c r="H14" s="1" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1542,11 +1566,11 @@
       <c r="F18" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G18" t="s">
-        <v>1</v>
-      </c>
-      <c r="H18" t="s">
-        <v>1</v>
+      <c r="G18" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1575,7 +1599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="187" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>108</v>
       </c>
@@ -1594,11 +1618,11 @@
       <c r="F20" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="G20" t="s">
-        <v>1</v>
-      </c>
-      <c r="H20" t="s">
-        <v>1</v>
+      <c r="G20" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1627,7 +1651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>117</v>
       </c>
@@ -1646,11 +1670,11 @@
       <c r="F22" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="G22" t="s">
-        <v>1</v>
-      </c>
-      <c r="H22" t="s">
-        <v>1</v>
+      <c r="G22" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1672,11 +1696,11 @@
       <c r="F23" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="G23" t="s">
-        <v>1</v>
-      </c>
-      <c r="H23" t="s">
-        <v>1</v>
+      <c r="G23" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1698,14 +1722,14 @@
       <c r="F24" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G24" t="s">
-        <v>1</v>
+      <c r="G24" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="H24" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>132</v>
       </c>
@@ -1724,11 +1748,11 @@
       <c r="F25" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="G25" t="s">
-        <v>1</v>
-      </c>
-      <c r="H25" t="s">
-        <v>1</v>
+      <c r="G25" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1891,7 +1915,7 @@
   <autoFilter ref="A1:H31" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H1 A4:H9 A2:F2 H2 A3:F3 A11:H11 A10:F10 A13:H31 A12:D12 F12 H12" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H1 A4:H6 A2:F2 H2 A3:F3 A11:F11 A10:F10 A13:F13 A12:D12 F12 H12 A26:H31 A23:F23 A19:H19 A18:D18 A15:H17 A14:G14 F18 A21:H21 A20:F20 A22:F22 H13 H11 A9:F9 H9 A8:F8 A7:F7 H7 A24:F24 H24 A25:F25" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>